<commit_message>
feat: publish detailed Horus-style teaching guide
</commit_message>
<xml_diff>
--- a/course/dist/04-09-2026-Lich-hoc-va-quan-ly-cohort-AI.xlsx
+++ b/course/dist/04-09-2026-Lich-hoc-va-quan-ly-cohort-AI.xlsx
@@ -3846,7 +3846,7 @@
       </c>
       <c r="B5" s="3" t="inlineStr">
         <is>
-          <t>Giáo án đầy đủ 6 tuần</t>
+          <t>Giáo án chi tiết Horus 6 tuần</t>
         </is>
       </c>
       <c r="C5" s="3" t="inlineStr">
@@ -3856,12 +3856,12 @@
       </c>
       <c r="D5" s="3" t="inlineStr">
         <is>
-          <t>PDF</t>
+          <t>DOCX/PDF</t>
         </is>
       </c>
       <c r="E5" s="3" t="inlineStr">
         <is>
-          <t>course/dist/04-09-2026-Giao-an-AI-Van-hanh-doanh-nghiep.pdf</t>
+          <t>course/dist/04-09-2026-Giao-an-chi-tiet-Horus-AI-Van-hanh-doanh-nghiep.pdf</t>
         </is>
       </c>
       <c r="F5" s="3" t="inlineStr">
@@ -3871,7 +3871,7 @@
       </c>
       <c r="G5" s="3" t="inlineStr">
         <is>
-          <t>Không phát toàn bộ nội bộ</t>
+          <t>Bản PDF để dạy; DOCX để chỉnh sửa</t>
         </is>
       </c>
     </row>

</xml_diff>